<commit_message>
modified:   backend/.env.example 	modified:   backend/api/report_templates/report_of_collections_and_deposits.xlsx 	new file:   backend/api/sms/__init__.py 	new file:   backend/api/sms/__pycache__/__init__.cpython-314.pyc 	new file:   backend/api/sms/__pycache__/semaphore.cpython-314.pyc 	new file:   backend/api/sms/semaphore.py 	modified:   backend/api/views/__pycache__/records.cpython-314.pyc 	modified:   backend/api/views/records.py 	modified:   backend/backend/__pycache__/settings.cpython-314.pyc 	modified:   backend/backend/settings.py 	modified:   backend/db_production.sqlite3 	modified:   backend/sync.log.1 	new file:   backend/sync.log.2 	modified:   src/app/dashboard/Dashboard.jsx 	modified:   src/pages/PublicView.jsx
</commit_message>
<xml_diff>
--- a/backend/api/report_templates/report_of_collections_and_deposits.xlsx
+++ b/backend/api/report_templates/report_of_collections_and_deposits.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\OneDrive\Desktop\New-folder-main (1) - Copy\iTURNO_capstone project\backend\api\report_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E086559B-4D3E-4C91-82E6-EEC48416AFE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37421D90-0483-4B43-824F-3942D2D7BE21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{C0A5B676-AB91-4A97-80CB-54385996E175}"/>
   </bookViews>
@@ -471,9 +471,111 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -498,10 +600,16 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -510,121 +618,13 @@
     <xf numFmtId="165" fontId="3" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -975,28 +975,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="54" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30"/>
-      <c r="H1" s="30"/>
+      <c r="B1" s="54"/>
+      <c r="C1" s="54"/>
+      <c r="D1" s="54"/>
+      <c r="E1" s="54"/>
+      <c r="F1" s="54"/>
+      <c r="G1" s="54"/>
+      <c r="H1" s="54"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="54" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
+      <c r="B2" s="54"/>
+      <c r="C2" s="54"/>
+      <c r="D2" s="54"/>
+      <c r="E2" s="54"/>
+      <c r="F2" s="54"/>
+      <c r="G2" s="54"/>
+      <c r="H2" s="54"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="21" t="s">
@@ -1015,10 +1015,10 @@
       <c r="H4" s="24"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="52" t="s">
+      <c r="A5" s="80" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="53"/>
+      <c r="B5" s="81"/>
       <c r="C5" s="25"/>
       <c r="D5" s="22"/>
       <c r="E5" s="25"/>
@@ -1039,10 +1039,10 @@
       <c r="H6" s="11"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="36" t="s">
+      <c r="A7" s="70" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="32" t="s">
+      <c r="B7" s="66" t="s">
         <v>5</v>
       </c>
       <c r="C7" s="2"/>
@@ -1053,8 +1053,8 @@
       <c r="H7" s="9"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="37"/>
-      <c r="B8" s="34"/>
+      <c r="A8" s="71"/>
+      <c r="B8" s="68"/>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -1075,295 +1075,295 @@
       <c r="H9" s="24"/>
     </row>
     <row r="10" spans="1:8" s="19" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="50" t="s">
+      <c r="A10" s="60" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="50"/>
-      <c r="C10" s="54" t="s">
+      <c r="B10" s="60"/>
+      <c r="C10" s="56" t="s">
         <v>31</v>
       </c>
-      <c r="D10" s="56"/>
-      <c r="E10" s="56"/>
-      <c r="F10" s="56"/>
-      <c r="G10" s="57" t="s">
+      <c r="D10" s="57"/>
+      <c r="E10" s="57"/>
+      <c r="F10" s="57"/>
+      <c r="G10" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="H10" s="58"/>
+      <c r="H10" s="34"/>
     </row>
     <row r="11" spans="1:8" s="19" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="50"/>
-      <c r="B11" s="50"/>
-      <c r="C11" s="54" t="s">
+      <c r="A11" s="60"/>
+      <c r="B11" s="60"/>
+      <c r="C11" s="56" t="s">
         <v>32</v>
       </c>
-      <c r="D11" s="55"/>
-      <c r="E11" s="54" t="s">
+      <c r="D11" s="58"/>
+      <c r="E11" s="56" t="s">
         <v>33</v>
       </c>
-      <c r="F11" s="55"/>
-      <c r="G11" s="59"/>
-      <c r="H11" s="60"/>
+      <c r="F11" s="58"/>
+      <c r="G11" s="35"/>
+      <c r="H11" s="37"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" s="51" t="s">
+      <c r="A12" s="82" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="51"/>
-      <c r="C12" s="47"/>
-      <c r="D12" s="48"/>
-      <c r="E12" s="39"/>
-      <c r="F12" s="40"/>
-      <c r="G12" s="39"/>
-      <c r="H12" s="40"/>
+      <c r="B12" s="82"/>
+      <c r="C12" s="75"/>
+      <c r="D12" s="76"/>
+      <c r="E12" s="63"/>
+      <c r="F12" s="64"/>
+      <c r="G12" s="63"/>
+      <c r="H12" s="64"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A13" s="51" t="s">
+      <c r="A13" s="82" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="51"/>
-      <c r="C13" s="47"/>
-      <c r="D13" s="48"/>
-      <c r="E13" s="39"/>
-      <c r="F13" s="40"/>
-      <c r="G13" s="39"/>
-      <c r="H13" s="40"/>
+      <c r="B13" s="82"/>
+      <c r="C13" s="75"/>
+      <c r="D13" s="76"/>
+      <c r="E13" s="63"/>
+      <c r="F13" s="64"/>
+      <c r="G13" s="63"/>
+      <c r="H13" s="64"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A14" s="51" t="s">
+      <c r="A14" s="82" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="51"/>
-      <c r="C14" s="47"/>
-      <c r="D14" s="48"/>
-      <c r="E14" s="39"/>
-      <c r="F14" s="40"/>
-      <c r="G14" s="39"/>
-      <c r="H14" s="40"/>
+      <c r="B14" s="82"/>
+      <c r="C14" s="75"/>
+      <c r="D14" s="76"/>
+      <c r="E14" s="63"/>
+      <c r="F14" s="64"/>
+      <c r="G14" s="63"/>
+      <c r="H14" s="64"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A15" s="51" t="s">
+      <c r="A15" s="82" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="51"/>
-      <c r="C15" s="47"/>
-      <c r="D15" s="48"/>
-      <c r="E15" s="39"/>
-      <c r="F15" s="40"/>
-      <c r="G15" s="39"/>
-      <c r="H15" s="40"/>
+      <c r="B15" s="82"/>
+      <c r="C15" s="75"/>
+      <c r="D15" s="76"/>
+      <c r="E15" s="63"/>
+      <c r="F15" s="64"/>
+      <c r="G15" s="63"/>
+      <c r="H15" s="64"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" s="29"/>
       <c r="B16" s="29"/>
-      <c r="C16" s="47"/>
-      <c r="D16" s="48"/>
-      <c r="E16" s="39"/>
-      <c r="F16" s="40"/>
-      <c r="G16" s="39"/>
-      <c r="H16" s="40"/>
+      <c r="C16" s="75"/>
+      <c r="D16" s="76"/>
+      <c r="E16" s="63"/>
+      <c r="F16" s="64"/>
+      <c r="G16" s="63"/>
+      <c r="H16" s="64"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="29"/>
       <c r="B17" s="29"/>
-      <c r="C17" s="47"/>
-      <c r="D17" s="48"/>
-      <c r="E17" s="39"/>
-      <c r="F17" s="40"/>
-      <c r="G17" s="39"/>
-      <c r="H17" s="40"/>
+      <c r="C17" s="75"/>
+      <c r="D17" s="76"/>
+      <c r="E17" s="63"/>
+      <c r="F17" s="64"/>
+      <c r="G17" s="63"/>
+      <c r="H17" s="64"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" s="29"/>
       <c r="B18" s="29"/>
-      <c r="C18" s="47"/>
-      <c r="D18" s="48"/>
-      <c r="E18" s="39"/>
-      <c r="F18" s="40"/>
-      <c r="G18" s="39"/>
-      <c r="H18" s="40"/>
+      <c r="C18" s="75"/>
+      <c r="D18" s="76"/>
+      <c r="E18" s="63"/>
+      <c r="F18" s="64"/>
+      <c r="G18" s="63"/>
+      <c r="H18" s="64"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="29"/>
       <c r="B19" s="29"/>
-      <c r="C19" s="47"/>
-      <c r="D19" s="48"/>
-      <c r="E19" s="39"/>
-      <c r="F19" s="40"/>
-      <c r="G19" s="39"/>
-      <c r="H19" s="40"/>
+      <c r="C19" s="75"/>
+      <c r="D19" s="76"/>
+      <c r="E19" s="63"/>
+      <c r="F19" s="64"/>
+      <c r="G19" s="63"/>
+      <c r="H19" s="64"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="29"/>
       <c r="B20" s="29"/>
-      <c r="C20" s="47"/>
-      <c r="D20" s="48"/>
-      <c r="E20" s="39"/>
-      <c r="F20" s="40"/>
-      <c r="G20" s="39"/>
-      <c r="H20" s="40"/>
+      <c r="C20" s="75"/>
+      <c r="D20" s="76"/>
+      <c r="E20" s="63"/>
+      <c r="F20" s="64"/>
+      <c r="G20" s="63"/>
+      <c r="H20" s="64"/>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" s="29"/>
       <c r="B21" s="29"/>
-      <c r="C21" s="47"/>
-      <c r="D21" s="48"/>
-      <c r="E21" s="39"/>
-      <c r="F21" s="40"/>
-      <c r="G21" s="39"/>
-      <c r="H21" s="40"/>
+      <c r="C21" s="75"/>
+      <c r="D21" s="76"/>
+      <c r="E21" s="63"/>
+      <c r="F21" s="64"/>
+      <c r="G21" s="63"/>
+      <c r="H21" s="64"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" s="29"/>
       <c r="B22" s="29"/>
-      <c r="C22" s="47"/>
-      <c r="D22" s="48"/>
-      <c r="E22" s="39"/>
-      <c r="F22" s="40"/>
-      <c r="G22" s="39"/>
-      <c r="H22" s="40"/>
+      <c r="C22" s="75"/>
+      <c r="D22" s="76"/>
+      <c r="E22" s="63"/>
+      <c r="F22" s="64"/>
+      <c r="G22" s="63"/>
+      <c r="H22" s="64"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="29"/>
       <c r="B23" s="29"/>
-      <c r="C23" s="47"/>
-      <c r="D23" s="48"/>
-      <c r="E23" s="39"/>
-      <c r="F23" s="40"/>
-      <c r="G23" s="39"/>
-      <c r="H23" s="40"/>
+      <c r="C23" s="75"/>
+      <c r="D23" s="76"/>
+      <c r="E23" s="63"/>
+      <c r="F23" s="64"/>
+      <c r="G23" s="63"/>
+      <c r="H23" s="64"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" s="29"/>
       <c r="B24" s="29"/>
-      <c r="C24" s="47"/>
-      <c r="D24" s="48"/>
-      <c r="E24" s="39"/>
-      <c r="F24" s="40"/>
-      <c r="G24" s="39"/>
-      <c r="H24" s="40"/>
+      <c r="C24" s="75"/>
+      <c r="D24" s="76"/>
+      <c r="E24" s="63"/>
+      <c r="F24" s="64"/>
+      <c r="G24" s="63"/>
+      <c r="H24" s="64"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="29"/>
       <c r="B25" s="29"/>
-      <c r="C25" s="47"/>
-      <c r="D25" s="48"/>
-      <c r="E25" s="39"/>
-      <c r="F25" s="40"/>
-      <c r="G25" s="39"/>
-      <c r="H25" s="40"/>
+      <c r="C25" s="75"/>
+      <c r="D25" s="76"/>
+      <c r="E25" s="63"/>
+      <c r="F25" s="64"/>
+      <c r="G25" s="63"/>
+      <c r="H25" s="64"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" s="29"/>
       <c r="B26" s="29"/>
-      <c r="C26" s="47"/>
-      <c r="D26" s="48"/>
-      <c r="E26" s="39"/>
-      <c r="F26" s="40"/>
-      <c r="G26" s="39"/>
-      <c r="H26" s="40"/>
+      <c r="C26" s="75"/>
+      <c r="D26" s="76"/>
+      <c r="E26" s="63"/>
+      <c r="F26" s="64"/>
+      <c r="G26" s="63"/>
+      <c r="H26" s="64"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" s="29"/>
       <c r="B27" s="29"/>
-      <c r="C27" s="47"/>
-      <c r="D27" s="48"/>
-      <c r="E27" s="39"/>
-      <c r="F27" s="40"/>
-      <c r="G27" s="39"/>
-      <c r="H27" s="40"/>
+      <c r="C27" s="75"/>
+      <c r="D27" s="76"/>
+      <c r="E27" s="63"/>
+      <c r="F27" s="64"/>
+      <c r="G27" s="63"/>
+      <c r="H27" s="64"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" s="29"/>
       <c r="B28" s="29"/>
-      <c r="C28" s="47"/>
-      <c r="D28" s="48"/>
-      <c r="E28" s="39"/>
-      <c r="F28" s="40"/>
-      <c r="G28" s="39"/>
-      <c r="H28" s="40"/>
+      <c r="C28" s="75"/>
+      <c r="D28" s="76"/>
+      <c r="E28" s="63"/>
+      <c r="F28" s="64"/>
+      <c r="G28" s="63"/>
+      <c r="H28" s="64"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" s="29"/>
       <c r="B29" s="29"/>
-      <c r="C29" s="47"/>
-      <c r="D29" s="48"/>
-      <c r="E29" s="39"/>
-      <c r="F29" s="40"/>
-      <c r="G29" s="39"/>
-      <c r="H29" s="40"/>
+      <c r="C29" s="75"/>
+      <c r="D29" s="76"/>
+      <c r="E29" s="63"/>
+      <c r="F29" s="64"/>
+      <c r="G29" s="63"/>
+      <c r="H29" s="64"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" s="29"/>
       <c r="B30" s="29"/>
-      <c r="C30" s="47"/>
-      <c r="D30" s="48"/>
-      <c r="E30" s="39"/>
-      <c r="F30" s="40"/>
-      <c r="G30" s="39"/>
-      <c r="H30" s="40"/>
+      <c r="C30" s="75"/>
+      <c r="D30" s="76"/>
+      <c r="E30" s="63"/>
+      <c r="F30" s="64"/>
+      <c r="G30" s="63"/>
+      <c r="H30" s="64"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" s="29"/>
       <c r="B31" s="29"/>
-      <c r="C31" s="47"/>
-      <c r="D31" s="48"/>
-      <c r="E31" s="39"/>
-      <c r="F31" s="40"/>
-      <c r="G31" s="39"/>
-      <c r="H31" s="40"/>
+      <c r="C31" s="75"/>
+      <c r="D31" s="76"/>
+      <c r="E31" s="63"/>
+      <c r="F31" s="64"/>
+      <c r="G31" s="63"/>
+      <c r="H31" s="64"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" s="29"/>
       <c r="B32" s="29"/>
-      <c r="C32" s="47"/>
-      <c r="D32" s="48"/>
-      <c r="E32" s="39"/>
-      <c r="F32" s="40"/>
-      <c r="G32" s="39"/>
-      <c r="H32" s="40"/>
+      <c r="C32" s="75"/>
+      <c r="D32" s="76"/>
+      <c r="E32" s="63"/>
+      <c r="F32" s="64"/>
+      <c r="G32" s="63"/>
+      <c r="H32" s="64"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A33" s="49" t="s">
+      <c r="A33" s="79" t="s">
         <v>14</v>
       </c>
-      <c r="B33" s="49"/>
-      <c r="C33" s="41">
+      <c r="B33" s="79"/>
+      <c r="C33" s="77">
         <f>SUM(C12:D32)</f>
         <v>0</v>
       </c>
-      <c r="D33" s="42"/>
-      <c r="E33" s="41">
+      <c r="D33" s="78"/>
+      <c r="E33" s="77">
         <f>SUM(E12:F32)</f>
         <v>0</v>
       </c>
-      <c r="F33" s="42"/>
-      <c r="G33" s="43">
+      <c r="F33" s="78"/>
+      <c r="G33" s="73">
         <f>SUM(G12:H32)</f>
         <v>0</v>
       </c>
-      <c r="H33" s="44"/>
+      <c r="H33" s="74"/>
     </row>
     <row r="34" spans="1:8" s="19" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A34" s="21"/>
-      <c r="B34" s="32" t="s">
+      <c r="B34" s="66" t="s">
         <v>16</v>
       </c>
-      <c r="C34" s="32"/>
-      <c r="D34" s="32"/>
-      <c r="E34" s="32"/>
-      <c r="F34" s="32"/>
-      <c r="G34" s="32"/>
-      <c r="H34" s="33"/>
+      <c r="C34" s="66"/>
+      <c r="D34" s="66"/>
+      <c r="E34" s="66"/>
+      <c r="F34" s="66"/>
+      <c r="G34" s="66"/>
+      <c r="H34" s="67"/>
     </row>
     <row r="35" spans="1:8" s="19" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A35" s="28"/>
-      <c r="B35" s="34"/>
-      <c r="C35" s="34"/>
-      <c r="D35" s="34"/>
-      <c r="E35" s="34"/>
-      <c r="F35" s="34"/>
-      <c r="G35" s="34"/>
-      <c r="H35" s="35"/>
+      <c r="B35" s="68"/>
+      <c r="C35" s="68"/>
+      <c r="D35" s="68"/>
+      <c r="E35" s="68"/>
+      <c r="F35" s="68"/>
+      <c r="G35" s="68"/>
+      <c r="H35" s="69"/>
     </row>
     <row r="36" spans="1:8" s="19" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A36" s="27" t="s">
@@ -1372,14 +1372,14 @@
       <c r="B36" s="22"/>
       <c r="C36" s="22"/>
       <c r="D36" s="22"/>
-      <c r="E36" s="45" t="s">
+      <c r="E36" s="51" t="s">
         <v>18</v>
       </c>
-      <c r="F36" s="46"/>
-      <c r="G36" s="45" t="s">
+      <c r="F36" s="53"/>
+      <c r="G36" s="51" t="s">
         <v>19</v>
       </c>
-      <c r="H36" s="46"/>
+      <c r="H36" s="53"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A37" s="29"/>
@@ -1502,44 +1502,44 @@
       <c r="H48" s="29"/>
     </row>
     <row r="49" spans="1:8" s="19" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="36" t="s">
+      <c r="A49" s="70" t="s">
         <v>21</v>
       </c>
-      <c r="B49" s="32" t="s">
+      <c r="B49" s="66" t="s">
         <v>20</v>
       </c>
-      <c r="C49" s="32"/>
-      <c r="D49" s="32"/>
-      <c r="E49" s="32"/>
-      <c r="F49" s="32"/>
-      <c r="G49" s="32"/>
-      <c r="H49" s="33"/>
+      <c r="C49" s="66"/>
+      <c r="D49" s="66"/>
+      <c r="E49" s="66"/>
+      <c r="F49" s="66"/>
+      <c r="G49" s="66"/>
+      <c r="H49" s="67"/>
     </row>
     <row r="50" spans="1:8" s="19" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="37"/>
-      <c r="B50" s="34"/>
-      <c r="C50" s="34"/>
-      <c r="D50" s="34"/>
-      <c r="E50" s="34"/>
-      <c r="F50" s="34"/>
-      <c r="G50" s="34"/>
-      <c r="H50" s="35"/>
+      <c r="A50" s="71"/>
+      <c r="B50" s="68"/>
+      <c r="C50" s="68"/>
+      <c r="D50" s="68"/>
+      <c r="E50" s="68"/>
+      <c r="F50" s="68"/>
+      <c r="G50" s="68"/>
+      <c r="H50" s="69"/>
     </row>
     <row r="51" spans="1:8" s="19" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="38" t="s">
+      <c r="A51" s="72" t="s">
         <v>25</v>
       </c>
-      <c r="B51" s="38"/>
-      <c r="C51" s="38"/>
-      <c r="D51" s="38"/>
-      <c r="E51" s="38" t="s">
+      <c r="B51" s="72"/>
+      <c r="C51" s="72"/>
+      <c r="D51" s="72"/>
+      <c r="E51" s="72" t="s">
         <v>22</v>
       </c>
-      <c r="F51" s="38"/>
-      <c r="G51" s="36" t="s">
+      <c r="F51" s="72"/>
+      <c r="G51" s="70" t="s">
         <v>19</v>
       </c>
-      <c r="H51" s="33"/>
+      <c r="H51" s="67"/>
     </row>
     <row r="52" spans="1:8" s="19" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A52" s="27"/>
@@ -1550,8 +1550,8 @@
         <v>23</v>
       </c>
       <c r="F52" s="21"/>
-      <c r="G52" s="37"/>
-      <c r="H52" s="35"/>
+      <c r="G52" s="71"/>
+      <c r="H52" s="69"/>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A53" s="10"/>
@@ -1668,12 +1668,12 @@
       <c r="H62" s="6"/>
     </row>
     <row r="63" spans="1:8" s="19" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="31" t="s">
+      <c r="A63" s="65" t="s">
         <v>26</v>
       </c>
-      <c r="B63" s="31"/>
-      <c r="C63" s="31"/>
-      <c r="D63" s="31"/>
+      <c r="B63" s="65"/>
+      <c r="C63" s="65"/>
+      <c r="D63" s="65"/>
       <c r="E63" s="14"/>
       <c r="F63" s="14"/>
       <c r="G63" s="14"/>
@@ -1684,9 +1684,13 @@
     </row>
   </sheetData>
   <mergeCells count="143">
-    <mergeCell ref="G14:H14"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="E12:F12"/>
     <mergeCell ref="A7:A8"/>
     <mergeCell ref="B7:B8"/>
     <mergeCell ref="A5:B5"/>
@@ -1701,12 +1705,6 @@
     <mergeCell ref="A10:B11"/>
     <mergeCell ref="A12:B12"/>
     <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="C16:D16"/>
     <mergeCell ref="A17:B17"/>
     <mergeCell ref="G17:H17"/>
     <mergeCell ref="E27:F27"/>
@@ -1725,6 +1723,12 @@
     <mergeCell ref="C20:D20"/>
     <mergeCell ref="C21:D21"/>
     <mergeCell ref="C22:D22"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="G23:H23"/>
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="E22:F22"/>
     <mergeCell ref="A32:B32"/>
     <mergeCell ref="A33:B33"/>
     <mergeCell ref="B34:H35"/>
@@ -1740,7 +1744,8 @@
     <mergeCell ref="A29:B29"/>
     <mergeCell ref="C28:D28"/>
     <mergeCell ref="C29:D29"/>
-    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="E28:F28"/>
+    <mergeCell ref="E29:F29"/>
     <mergeCell ref="E13:F13"/>
     <mergeCell ref="E14:F14"/>
     <mergeCell ref="E15:F15"/>
@@ -1751,39 +1756,29 @@
     <mergeCell ref="C19:D19"/>
     <mergeCell ref="G18:H18"/>
     <mergeCell ref="G19:H19"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="G23:H23"/>
-    <mergeCell ref="E28:F28"/>
-    <mergeCell ref="E29:F29"/>
-    <mergeCell ref="E21:F21"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="E25:F25"/>
-    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="G16:H16"/>
     <mergeCell ref="C30:D30"/>
     <mergeCell ref="C31:D31"/>
     <mergeCell ref="C32:D32"/>
     <mergeCell ref="C33:D33"/>
     <mergeCell ref="G37:H37"/>
-    <mergeCell ref="G38:H38"/>
-    <mergeCell ref="G24:H24"/>
-    <mergeCell ref="G25:H25"/>
-    <mergeCell ref="G26:H26"/>
-    <mergeCell ref="G27:H27"/>
+    <mergeCell ref="E33:F33"/>
+    <mergeCell ref="E36:F36"/>
+    <mergeCell ref="E30:F30"/>
+    <mergeCell ref="E31:F31"/>
+    <mergeCell ref="E32:F32"/>
     <mergeCell ref="G28:H28"/>
     <mergeCell ref="G29:H29"/>
     <mergeCell ref="G31:H31"/>
     <mergeCell ref="G32:H32"/>
-    <mergeCell ref="E33:F33"/>
     <mergeCell ref="G33:H33"/>
-    <mergeCell ref="E36:F36"/>
     <mergeCell ref="G36:H36"/>
-    <mergeCell ref="E30:F30"/>
-    <mergeCell ref="E31:F31"/>
-    <mergeCell ref="E32:F32"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="E26:F26"/>
     <mergeCell ref="A63:D63"/>
     <mergeCell ref="E48:F48"/>
     <mergeCell ref="G48:H48"/>
@@ -1827,6 +1822,11 @@
     <mergeCell ref="A40:D40"/>
     <mergeCell ref="A41:D41"/>
     <mergeCell ref="G30:H30"/>
+    <mergeCell ref="G38:H38"/>
+    <mergeCell ref="G24:H24"/>
+    <mergeCell ref="G25:H25"/>
+    <mergeCell ref="G26:H26"/>
+    <mergeCell ref="G27:H27"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="78" fitToHeight="0" orientation="portrait" r:id="rId1"/>
@@ -1852,61 +1852,61 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="54" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30"/>
-      <c r="H1" s="30"/>
-      <c r="I1" s="30"/>
-      <c r="J1" s="30"/>
-      <c r="K1" s="30"/>
-      <c r="L1" s="30"/>
-      <c r="M1" s="30"/>
+      <c r="B1" s="54"/>
+      <c r="C1" s="54"/>
+      <c r="D1" s="54"/>
+      <c r="E1" s="54"/>
+      <c r="F1" s="54"/>
+      <c r="G1" s="54"/>
+      <c r="H1" s="54"/>
+      <c r="I1" s="54"/>
+      <c r="J1" s="54"/>
+      <c r="K1" s="54"/>
+      <c r="L1" s="54"/>
+      <c r="M1" s="54"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="54" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
-      <c r="I2" s="30"/>
-      <c r="J2" s="30"/>
-      <c r="K2" s="30"/>
-      <c r="L2" s="30"/>
-      <c r="M2" s="30"/>
+      <c r="B2" s="54"/>
+      <c r="C2" s="54"/>
+      <c r="D2" s="54"/>
+      <c r="E2" s="54"/>
+      <c r="F2" s="54"/>
+      <c r="G2" s="54"/>
+      <c r="H2" s="54"/>
+      <c r="I2" s="54"/>
+      <c r="J2" s="54"/>
+      <c r="K2" s="54"/>
+      <c r="L2" s="54"/>
+      <c r="M2" s="54"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A3" s="80"/>
-      <c r="B3" s="80"/>
-      <c r="C3" s="80"/>
-      <c r="D3" s="80"/>
-      <c r="E3" s="80"/>
-      <c r="F3" s="80"/>
-      <c r="G3" s="80"/>
-      <c r="H3" s="80"/>
-      <c r="I3" s="80"/>
-      <c r="J3" s="80"/>
-      <c r="K3" s="80"/>
-      <c r="L3" s="80"/>
-      <c r="M3" s="80"/>
+      <c r="A3" s="59"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="59"/>
+      <c r="G3" s="59"/>
+      <c r="H3" s="59"/>
+      <c r="I3" s="59"/>
+      <c r="J3" s="59"/>
+      <c r="K3" s="59"/>
+      <c r="L3" s="59"/>
+      <c r="M3" s="59"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A4" s="45" t="s">
+      <c r="A4" s="51" t="s">
         <v>27</v>
       </c>
-      <c r="B4" s="78"/>
-      <c r="C4" s="78"/>
-      <c r="D4" s="78"/>
+      <c r="B4" s="52"/>
+      <c r="C4" s="52"/>
+      <c r="D4" s="52"/>
       <c r="E4" s="5"/>
       <c r="F4" s="5"/>
       <c r="G4" s="5"/>
@@ -1918,54 +1918,54 @@
       <c r="M4" s="7"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A5" s="82" t="s">
+      <c r="A5" s="62" t="s">
         <v>28</v>
       </c>
-      <c r="B5" s="54" t="s">
+      <c r="B5" s="56" t="s">
         <v>29</v>
       </c>
-      <c r="C5" s="56"/>
-      <c r="D5" s="55"/>
-      <c r="E5" s="54" t="s">
+      <c r="C5" s="57"/>
+      <c r="D5" s="58"/>
+      <c r="E5" s="56" t="s">
         <v>34</v>
       </c>
-      <c r="F5" s="56"/>
-      <c r="G5" s="55"/>
-      <c r="H5" s="54" t="s">
+      <c r="F5" s="57"/>
+      <c r="G5" s="58"/>
+      <c r="H5" s="56" t="s">
         <v>35</v>
       </c>
-      <c r="I5" s="56"/>
-      <c r="J5" s="55"/>
-      <c r="K5" s="54" t="s">
+      <c r="I5" s="57"/>
+      <c r="J5" s="58"/>
+      <c r="K5" s="56" t="s">
         <v>36</v>
       </c>
-      <c r="L5" s="56"/>
-      <c r="M5" s="55"/>
+      <c r="L5" s="57"/>
+      <c r="M5" s="58"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A6" s="50"/>
-      <c r="B6" s="50" t="s">
+      <c r="A6" s="60"/>
+      <c r="B6" s="60" t="s">
         <v>30</v>
       </c>
       <c r="C6" s="29" t="s">
         <v>31</v>
       </c>
       <c r="D6" s="29"/>
-      <c r="E6" s="50" t="s">
+      <c r="E6" s="60" t="s">
         <v>30</v>
       </c>
       <c r="F6" s="29" t="s">
         <v>31</v>
       </c>
       <c r="G6" s="29"/>
-      <c r="H6" s="50" t="s">
+      <c r="H6" s="60" t="s">
         <v>30</v>
       </c>
       <c r="I6" s="29" t="s">
         <v>31</v>
       </c>
       <c r="J6" s="29"/>
-      <c r="K6" s="50" t="s">
+      <c r="K6" s="60" t="s">
         <v>30</v>
       </c>
       <c r="L6" s="29" t="s">
@@ -1974,29 +1974,29 @@
       <c r="M6" s="29"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A7" s="81"/>
-      <c r="B7" s="81"/>
+      <c r="A7" s="61"/>
+      <c r="B7" s="61"/>
       <c r="C7" s="16" t="s">
         <v>32</v>
       </c>
       <c r="D7" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="E7" s="81"/>
+      <c r="E7" s="61"/>
       <c r="F7" s="16" t="s">
         <v>32</v>
       </c>
       <c r="G7" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="H7" s="81"/>
+      <c r="H7" s="61"/>
       <c r="I7" s="16" t="s">
         <v>32</v>
       </c>
       <c r="J7" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="K7" s="81"/>
+      <c r="K7" s="61"/>
       <c r="L7" s="16" t="s">
         <v>32</v>
       </c>
@@ -2632,46 +2632,46 @@
         <v>26</v>
       </c>
       <c r="B49" s="6"/>
-      <c r="C49" s="75">
+      <c r="C49" s="48">
         <f>SUM(C8:D48)</f>
         <v>0</v>
       </c>
-      <c r="D49" s="75"/>
+      <c r="D49" s="48"/>
       <c r="E49" s="6"/>
-      <c r="F49" s="76">
+      <c r="F49" s="49">
         <f>SUM(F8:G48)</f>
         <v>0</v>
       </c>
-      <c r="G49" s="77"/>
+      <c r="G49" s="50"/>
       <c r="H49" s="6"/>
-      <c r="I49" s="75">
+      <c r="I49" s="48">
         <f>SUM(I8:J48)</f>
         <v>0</v>
       </c>
-      <c r="J49" s="75"/>
+      <c r="J49" s="48"/>
       <c r="K49" s="6"/>
-      <c r="L49" s="75">
+      <c r="L49" s="48">
         <f>SUM(L8:M48)</f>
         <v>0</v>
       </c>
-      <c r="M49" s="75"/>
+      <c r="M49" s="48"/>
     </row>
     <row r="50" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A50" s="45" t="s">
+      <c r="A50" s="51" t="s">
         <v>37</v>
       </c>
-      <c r="B50" s="78"/>
-      <c r="C50" s="78"/>
-      <c r="D50" s="78"/>
-      <c r="E50" s="78"/>
-      <c r="F50" s="78"/>
-      <c r="G50" s="78"/>
-      <c r="H50" s="78"/>
-      <c r="I50" s="78"/>
-      <c r="J50" s="78"/>
-      <c r="K50" s="78"/>
-      <c r="L50" s="78"/>
-      <c r="M50" s="46"/>
+      <c r="B50" s="52"/>
+      <c r="C50" s="52"/>
+      <c r="D50" s="52"/>
+      <c r="E50" s="52"/>
+      <c r="F50" s="52"/>
+      <c r="G50" s="52"/>
+      <c r="H50" s="52"/>
+      <c r="I50" s="52"/>
+      <c r="J50" s="52"/>
+      <c r="K50" s="52"/>
+      <c r="L50" s="52"/>
+      <c r="M50" s="53"/>
     </row>
     <row r="51" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A51" s="3" t="s">
@@ -2689,20 +2689,20 @@
       </c>
       <c r="H51" s="1"/>
       <c r="I51" s="1"/>
-      <c r="J51" s="79" t="s">
+      <c r="J51" s="55" t="s">
         <v>52</v>
       </c>
-      <c r="K51" s="79"/>
+      <c r="K51" s="55"/>
       <c r="M51" s="11"/>
     </row>
     <row r="52" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A52" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="J52" s="30" t="s">
+      <c r="J52" s="54" t="s">
         <v>55</v>
       </c>
-      <c r="K52" s="30"/>
+      <c r="K52" s="54"/>
       <c r="L52" s="19" t="s">
         <v>44</v>
       </c>
@@ -2787,62 +2787,62 @@
       <c r="M59" s="11"/>
     </row>
     <row r="60" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A60" s="73" t="s">
+      <c r="A60" s="46" t="s">
         <v>46</v>
       </c>
-      <c r="B60" s="73"/>
-      <c r="C60" s="73"/>
-      <c r="D60" s="73"/>
-      <c r="E60" s="74"/>
-      <c r="F60" s="68" t="s">
+      <c r="B60" s="46"/>
+      <c r="C60" s="46"/>
+      <c r="D60" s="46"/>
+      <c r="E60" s="47"/>
+      <c r="F60" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="G60" s="69"/>
-      <c r="H60" s="69"/>
-      <c r="I60" s="69"/>
-      <c r="J60" s="69"/>
-      <c r="K60" s="69"/>
-      <c r="L60" s="69"/>
-      <c r="M60" s="70"/>
+      <c r="G60" s="42"/>
+      <c r="H60" s="42"/>
+      <c r="I60" s="42"/>
+      <c r="J60" s="42"/>
+      <c r="K60" s="42"/>
+      <c r="L60" s="42"/>
+      <c r="M60" s="43"/>
     </row>
     <row r="61" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A61" s="73"/>
-      <c r="B61" s="73"/>
-      <c r="C61" s="73"/>
-      <c r="D61" s="73"/>
-      <c r="E61" s="73"/>
-      <c r="F61" s="71" t="s">
+      <c r="A61" s="46"/>
+      <c r="B61" s="46"/>
+      <c r="C61" s="46"/>
+      <c r="D61" s="46"/>
+      <c r="E61" s="46"/>
+      <c r="F61" s="44" t="s">
         <v>48</v>
       </c>
-      <c r="G61" s="71"/>
-      <c r="H61" s="71"/>
-      <c r="I61" s="71"/>
-      <c r="J61" s="71"/>
-      <c r="K61" s="71"/>
-      <c r="L61" s="71"/>
-      <c r="M61" s="71"/>
+      <c r="G61" s="44"/>
+      <c r="H61" s="44"/>
+      <c r="I61" s="44"/>
+      <c r="J61" s="44"/>
+      <c r="K61" s="44"/>
+      <c r="L61" s="44"/>
+      <c r="M61" s="44"/>
     </row>
     <row r="62" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A62" s="73"/>
-      <c r="B62" s="73"/>
-      <c r="C62" s="73"/>
-      <c r="D62" s="73"/>
-      <c r="E62" s="73"/>
-      <c r="F62" s="72"/>
-      <c r="G62" s="72"/>
-      <c r="H62" s="72"/>
-      <c r="I62" s="72"/>
-      <c r="J62" s="72"/>
-      <c r="K62" s="72"/>
-      <c r="L62" s="72"/>
-      <c r="M62" s="72"/>
+      <c r="A62" s="46"/>
+      <c r="B62" s="46"/>
+      <c r="C62" s="46"/>
+      <c r="D62" s="46"/>
+      <c r="E62" s="46"/>
+      <c r="F62" s="45"/>
+      <c r="G62" s="45"/>
+      <c r="H62" s="45"/>
+      <c r="I62" s="45"/>
+      <c r="J62" s="45"/>
+      <c r="K62" s="45"/>
+      <c r="L62" s="45"/>
+      <c r="M62" s="45"/>
     </row>
     <row r="63" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A63" s="73"/>
-      <c r="B63" s="73"/>
-      <c r="C63" s="73"/>
-      <c r="D63" s="73"/>
-      <c r="E63" s="73"/>
+      <c r="A63" s="46"/>
+      <c r="B63" s="46"/>
+      <c r="C63" s="46"/>
+      <c r="D63" s="46"/>
+      <c r="E63" s="46"/>
       <c r="F63" s="29"/>
       <c r="G63" s="29"/>
       <c r="H63" s="29"/>
@@ -2853,11 +2853,11 @@
       <c r="M63" s="29"/>
     </row>
     <row r="64" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A64" s="73"/>
-      <c r="B64" s="73"/>
-      <c r="C64" s="73"/>
-      <c r="D64" s="73"/>
-      <c r="E64" s="73"/>
+      <c r="A64" s="46"/>
+      <c r="B64" s="46"/>
+      <c r="C64" s="46"/>
+      <c r="D64" s="46"/>
+      <c r="E64" s="46"/>
       <c r="F64" s="29"/>
       <c r="G64" s="29"/>
       <c r="H64" s="29"/>
@@ -2868,59 +2868,59 @@
       <c r="M64" s="29"/>
     </row>
     <row r="65" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A65" s="65"/>
-      <c r="B65" s="67"/>
-      <c r="C65" s="66"/>
-      <c r="D65" s="65"/>
-      <c r="E65" s="66"/>
-      <c r="F65" s="61" t="s">
+      <c r="A65" s="38"/>
+      <c r="B65" s="40"/>
+      <c r="C65" s="39"/>
+      <c r="D65" s="38"/>
+      <c r="E65" s="39"/>
+      <c r="F65" s="30" t="s">
         <v>51</v>
       </c>
-      <c r="G65" s="61"/>
-      <c r="H65" s="61"/>
-      <c r="I65" s="61"/>
-      <c r="J65" s="61"/>
-      <c r="K65" s="61"/>
+      <c r="G65" s="30"/>
+      <c r="H65" s="30"/>
+      <c r="I65" s="30"/>
+      <c r="J65" s="30"/>
+      <c r="K65" s="30"/>
       <c r="L65" s="29"/>
       <c r="M65" s="29"/>
     </row>
     <row r="66" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A66" s="57" t="s">
+      <c r="A66" s="32" t="s">
         <v>49</v>
       </c>
-      <c r="B66" s="63"/>
-      <c r="C66" s="58"/>
-      <c r="D66" s="62" t="s">
+      <c r="B66" s="33"/>
+      <c r="C66" s="34"/>
+      <c r="D66" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="E66" s="62"/>
-      <c r="F66" s="62" t="s">
+      <c r="E66" s="31"/>
+      <c r="F66" s="31" t="s">
         <v>50</v>
       </c>
-      <c r="G66" s="62"/>
-      <c r="H66" s="62"/>
-      <c r="I66" s="62"/>
-      <c r="J66" s="62"/>
-      <c r="K66" s="62"/>
-      <c r="L66" s="62" t="s">
+      <c r="G66" s="31"/>
+      <c r="H66" s="31"/>
+      <c r="I66" s="31"/>
+      <c r="J66" s="31"/>
+      <c r="K66" s="31"/>
+      <c r="L66" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="M66" s="62"/>
+      <c r="M66" s="31"/>
     </row>
     <row r="67" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A67" s="59"/>
-      <c r="B67" s="64"/>
-      <c r="C67" s="60"/>
-      <c r="D67" s="62"/>
-      <c r="E67" s="62"/>
-      <c r="F67" s="62"/>
-      <c r="G67" s="62"/>
-      <c r="H67" s="62"/>
-      <c r="I67" s="62"/>
-      <c r="J67" s="62"/>
-      <c r="K67" s="62"/>
-      <c r="L67" s="62"/>
-      <c r="M67" s="62"/>
+      <c r="A67" s="35"/>
+      <c r="B67" s="36"/>
+      <c r="C67" s="37"/>
+      <c r="D67" s="31"/>
+      <c r="E67" s="31"/>
+      <c r="F67" s="31"/>
+      <c r="G67" s="31"/>
+      <c r="H67" s="31"/>
+      <c r="I67" s="31"/>
+      <c r="J67" s="31"/>
+      <c r="K67" s="31"/>
+      <c r="L67" s="31"/>
+      <c r="M67" s="31"/>
     </row>
   </sheetData>
   <mergeCells count="203">

</xml_diff>